<commit_message>
Atualiza progresso do aluno
</commit_message>
<xml_diff>
--- a/personal fit pro dashboard 3.xlsx
+++ b/personal fit pro dashboard 3.xlsx
@@ -2421,7 +2421,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="str">
@@ -2457,9 +2457,26 @@
         <v>2026-09-16T11:54:31.401Z</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="1" t="str">
+        <v>Yury</v>
+      </c>
+      <c r="B3" s="1" t="str">
+        <v>A</v>
+      </c>
+      <c r="C3" s="1">
+        <v>0</v>
+      </c>
+      <c r="D3" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="E3" s="1" t="str">
+        <v>2026-09-16T13:07:18.713Z</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>